<commit_message>
excel charts (without video)
</commit_message>
<xml_diff>
--- a/lastname_territory_chart.xlsx
+++ b/lastname_territory_chart.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
-  <workbookPr hidePivotFieldList="1" defaultThemeVersion="202300"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kasaiahantonio\Desktop\datalab\capstone1\Capstone_1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1DDD82BE-D18C-453E-8C73-35DD1B5D61A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B7579A16-368A-4D15-86C7-9E93BE8321D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{04C86A0B-4F46-4F01-BB47-7FAABC4FE2A4}"/>
+    <workbookView xWindow="-80" yWindow="-80" windowWidth="19360" windowHeight="11440" xr2:uid="{04C86A0B-4F46-4F01-BB47-7FAABC4FE2A4}"/>
   </bookViews>
   <sheets>
     <sheet name="capstone_file_export_query3" sheetId="1" r:id="rId1"/>
@@ -29,12 +29,6 @@
   </si>
   <si>
     <t>Territory</t>
-  </si>
-  <si>
-    <t>Territory_Revenue</t>
-  </si>
-  <si>
-    <t>Region_Revenue</t>
   </si>
   <si>
     <t>East</t>
@@ -85,10 +79,16 @@
     <t>Grand Total</t>
   </si>
   <si>
-    <t>Sum of Territory_Revenue</t>
+    <t>Territory Revenue</t>
   </si>
   <si>
-    <t>Sum of Region_Revenue</t>
+    <t>Region Revenue</t>
+  </si>
+  <si>
+    <t>Sum of Region Revenue</t>
+  </si>
+  <si>
+    <t>Sum of Territory Revenue</t>
   </si>
 </sst>
 </file>
@@ -2698,7 +2698,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Sum of Region_Revenue</c:v>
+                  <c:v>Sum of Region Revenue</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -2821,7 +2821,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Sum of Territory_Revenue</c:v>
+                  <c:v>Sum of Territory Revenue</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -3735,6 +3735,85 @@
     </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>6350</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>88900</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>12700</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>165100</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="3" name="TextBox 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4E209800-1E47-90BB-68B9-9468C8B0ED83}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4311650" y="88900"/>
+          <a:ext cx="5956300" cy="812800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0" i="0" cap="all">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Business Question : Provide a comparison of total revenue for the specific sales territory and the region it belongs to. </a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -3863,7 +3942,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E8288F3A-921D-449C-9CC9-EA32D4093814}" name="PivotTable2" cacheId="13" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E8288F3A-921D-449C-9CC9-EA32D4093814}" name="PivotTable2" cacheId="13" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="4">
   <location ref="I7:K22" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="4">
     <pivotField axis="axisRow" showAll="0">
@@ -3978,8 +4057,8 @@
     </i>
   </colItems>
   <dataFields count="2">
-    <dataField name="Sum of Region_Revenue" fld="3" baseField="1" baseItem="0"/>
-    <dataField name="Sum of Territory_Revenue" fld="2" baseField="0" baseItem="0"/>
+    <dataField name="Sum of Region Revenue" fld="3" baseField="0" baseItem="0"/>
+    <dataField name="Sum of Territory Revenue" fld="2" baseField="0" baseItem="0"/>
   </dataFields>
   <chartFormats count="12">
     <chartFormat chart="0" format="20" series="1">
@@ -4109,8 +4188,8 @@
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{8845B1E2-72AC-4BCE-9F2D-4AD591D7134B}" name="Region"/>
     <tableColumn id="2" xr3:uid="{9F2F51CD-51C2-4061-B1E1-3D07E34F23D7}" name="Territory"/>
-    <tableColumn id="3" xr3:uid="{7D7447DF-44E1-4A31-91AA-6E77717C0B6B}" name="Territory_Revenue"/>
-    <tableColumn id="4" xr3:uid="{6CF171D9-5E2C-4829-BB66-A09AC5B3D2BE}" name="Region_Revenue"/>
+    <tableColumn id="3" xr3:uid="{7D7447DF-44E1-4A31-91AA-6E77717C0B6B}" name="Territory Revenue"/>
+    <tableColumn id="4" xr3:uid="{6CF171D9-5E2C-4829-BB66-A09AC5B3D2BE}" name="Region Revenue"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4440,8 +4519,8 @@
     <col min="3" max="3" width="17.81640625" customWidth="1"/>
     <col min="4" max="4" width="16.6328125" customWidth="1"/>
     <col min="9" max="9" width="16.6328125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="21.08984375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="22.26953125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="20.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="21.81640625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="11.81640625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="10.81640625" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="22.26953125" bestFit="1" customWidth="1"/>
@@ -4463,18 +4542,18 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="D1" t="s">
-        <v>3</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C2">
         <v>2392222.44</v>
@@ -4485,10 +4564,10 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
         <v>4</v>
-      </c>
-      <c r="B3" t="s">
-        <v>6</v>
       </c>
       <c r="C3">
         <v>4330817.09</v>
@@ -4499,10 +4578,10 @@
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B4" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C4">
         <v>1877249.75</v>
@@ -4513,10 +4592,10 @@
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" t="s">
         <v>7</v>
-      </c>
-      <c r="B5" t="s">
-        <v>9</v>
       </c>
       <c r="C5">
         <v>11451615.09</v>
@@ -4527,10 +4606,10 @@
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C6">
         <v>5733256.2699999996</v>
@@ -4541,10 +4620,10 @@
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C7">
         <v>5175405.87</v>
@@ -4553,21 +4632,21 @@
         <v>24237526.98</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="J7" t="s">
+        <v>20</v>
+      </c>
+      <c r="K7" t="s">
         <v>21</v>
-      </c>
-      <c r="K7" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B8" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C8">
         <v>3930187.55</v>
@@ -4576,7 +4655,7 @@
         <v>7996850.1200000001</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J8" s="3">
         <v>13446079.060000001</v>
@@ -4587,10 +4666,10 @@
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" t="s">
         <v>12</v>
-      </c>
-      <c r="B9" t="s">
-        <v>14</v>
       </c>
       <c r="C9">
         <v>648812.56000000006</v>
@@ -4599,7 +4678,7 @@
         <v>7996850.1200000001</v>
       </c>
       <c r="I9" s="4" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J9" s="3">
         <v>6723039.5300000003</v>
@@ -4610,10 +4689,10 @@
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B10" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C10">
         <v>3417850.01</v>
@@ -4622,7 +4701,7 @@
         <v>7996850.1200000001</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J10" s="3">
         <v>6723039.5300000003</v>
@@ -4633,10 +4712,10 @@
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B11" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C11">
         <v>6412632.2199999997</v>
@@ -4645,7 +4724,7 @@
         <v>6412632.2199999997</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J11" s="3">
         <v>96950107.920000002</v>
@@ -4656,7 +4735,7 @@
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.35">
       <c r="I12" s="4" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="J12" s="3">
         <v>24237526.98</v>
@@ -4667,7 +4746,7 @@
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="I13" s="4" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="J13" s="3">
         <v>24237526.98</v>
@@ -4678,7 +4757,7 @@
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.35">
       <c r="I14" s="4" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="J14" s="3">
         <v>24237526.98</v>
@@ -4689,7 +4768,7 @@
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.35">
       <c r="I15" s="4" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="J15" s="3">
         <v>24237526.98</v>
@@ -4700,7 +4779,7 @@
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.35">
       <c r="I16" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="J16" s="3">
         <v>23990550.359999999</v>
@@ -4711,7 +4790,7 @@
     </row>
     <row r="17" spans="9:11" x14ac:dyDescent="0.35">
       <c r="I17" s="4" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="J17" s="3">
         <v>7996850.1200000001</v>
@@ -4722,7 +4801,7 @@
     </row>
     <row r="18" spans="9:11" x14ac:dyDescent="0.35">
       <c r="I18" s="4" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="J18" s="3">
         <v>7996850.1200000001</v>
@@ -4733,7 +4812,7 @@
     </row>
     <row r="19" spans="9:11" x14ac:dyDescent="0.35">
       <c r="I19" s="4" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="J19" s="3">
         <v>7996850.1200000001</v>
@@ -4744,7 +4823,7 @@
     </row>
     <row r="20" spans="9:11" x14ac:dyDescent="0.35">
       <c r="I20" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="J20" s="3">
         <v>6412632.2199999997</v>
@@ -4755,7 +4834,7 @@
     </row>
     <row r="21" spans="9:11" x14ac:dyDescent="0.35">
       <c r="I21" s="4" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="J21" s="3">
         <v>6412632.2199999997</v>
@@ -4766,7 +4845,7 @@
     </row>
     <row r="22" spans="9:11" x14ac:dyDescent="0.35">
       <c r="I22" s="2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="J22" s="3">
         <v>140799369.56</v>

</xml_diff>